<commit_message>
added many moves without rotations
</commit_message>
<xml_diff>
--- a/move map.xlsx
+++ b/move map.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chris/main/code/solve.training/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chris/main/code/solve.training.beta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33687C7F-3E9D-3143-9876-F39A5C7E416F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DBA2F1A-8D18-1E43-8043-8FA0B3CD6581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="640" windowWidth="30240" windowHeight="19000" xr2:uid="{967E5E10-9561-A846-A84D-E0929CE543E7}"/>
   </bookViews>
@@ -620,10 +620,10 @@
         <v>46</v>
       </c>
       <c r="F4" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H4" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="I4" t="s">
         <v>20</v>
@@ -748,10 +748,10 @@
         <v>21</v>
       </c>
       <c r="F10" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="H10" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="I10" t="s">
         <v>48</v>

</xml_diff>

<commit_message>
full cube play working
</commit_message>
<xml_diff>
--- a/move map.xlsx
+++ b/move map.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chris/main/code/solve.training.beta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DBA2F1A-8D18-1E43-8043-8FA0B3CD6581}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19378FAE-7FD7-7E42-88F8-0B11F87D825E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="640" windowWidth="30240" windowHeight="19000" xr2:uid="{967E5E10-9561-A846-A84D-E0929CE543E7}"/>
   </bookViews>
@@ -617,7 +617,7 @@
         <v>37</v>
       </c>
       <c r="E4" t="s">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="F4" t="s">
         <v>44</v>
@@ -745,7 +745,7 @@
         <v>50</v>
       </c>
       <c r="E10" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="F10" t="s">
         <v>40</v>

</xml_diff>